<commit_message>
Agregar indicador de última actualización en Slip Robots
</commit_message>
<xml_diff>
--- a/herramientas/data/sliprobots/slip_robots_datos.xlsx
+++ b/herramientas/data/sliprobots/slip_robots_datos.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -594,6 +594,18 @@
       <c r="B14" t="inlineStr">
         <is>
           <t>Incluyendo circuito PoC. Target largo plazo: 78%+</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ultima_actualizacion</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
         </is>
       </c>
     </row>

</xml_diff>